<commit_message>
Include non-duplicated items in warehouse and combined sheets
Warehouse sheets (倉庫別_*) and the combined sheet (商品別_合算) now
list every item, with a 区分 column (重複/単独), duplicate rows
highlighted, and subtotals for duplicated vs. single-location items.
Applied to both the 20260929DDD and 26.9 SAP workbooks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EvAM76XRuw9ucoZyZ3Azwt
</commit_message>
<xml_diff>
--- a/output/20260929DDD_SAP_重複商品集計.xlsx
+++ b/output/20260929DDD_SAP_重複商品集計.xlsx
@@ -5,14 +5,14 @@
   <sheets>
     <sheet name="XTab DS_1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Filter DS_1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="重複_CX催事" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="重複_DBS倉庫" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="重複商品_合算" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="倉庫別_CX催事" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="倉庫別_DBS倉庫" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="商品別_合算" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'重複_CX催事'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'重複_DBS倉庫'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'重複商品_合算'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'倉庫別_CX催事'!$A$1:$H$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'倉庫別_DBS倉庫'!$A$1:$H$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'商品別_合算'!$A$1:$K$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -60,7 +60,7 @@
       <color rgb="00595959"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -74,7 +74,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,14 +143,28 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -4304,7 +4328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="2" min="1" max="1"/>
@@ -4312,8 +4336,9 @@
     <col width="52" customWidth="1" style="2" min="3" max="3"/>
     <col width="10" customWidth="1" style="2" min="4" max="4"/>
     <col width="12" customWidth="1" style="2" min="5" max="5"/>
-    <col width="14" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
+    <col width="8" customWidth="1" style="2" min="6" max="6"/>
+    <col width="14" customWidth="1" style="2" min="7" max="7"/>
+    <col width="16" customWidth="1" style="2" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4344,10 +4369,15 @@
       </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
           <t>在庫数量</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>在庫金額</t>
         </is>
@@ -4380,10 +4410,14 @@
         </is>
       </c>
       <c r="F2" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B2)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G2" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B2,'XTab DS_1'!$D$2:$D$106,$D2)</f>
         <v/>
       </c>
-      <c r="G2" s="11">
+      <c r="H2" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B2,'XTab DS_1'!$D$2:$D$106,$D2)</f>
         <v/>
       </c>
@@ -4415,10 +4449,14 @@
         </is>
       </c>
       <c r="F3" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B3)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G3" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B3,'XTab DS_1'!$D$2:$D$106,$D3)</f>
         <v/>
       </c>
-      <c r="G3" s="11">
+      <c r="H3" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B3,'XTab DS_1'!$D$2:$D$106,$D3)</f>
         <v/>
       </c>
@@ -4450,10 +4488,14 @@
         </is>
       </c>
       <c r="F4" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B4)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G4" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B4,'XTab DS_1'!$D$2:$D$106,$D4)</f>
         <v/>
       </c>
-      <c r="G4" s="11">
+      <c r="H4" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B4,'XTab DS_1'!$D$2:$D$106,$D4)</f>
         <v/>
       </c>
@@ -4485,10 +4527,14 @@
         </is>
       </c>
       <c r="F5" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B5)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G5" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B5,'XTab DS_1'!$D$2:$D$106,$D5)</f>
         <v/>
       </c>
-      <c r="G5" s="11">
+      <c r="H5" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B5,'XTab DS_1'!$D$2:$D$106,$D5)</f>
         <v/>
       </c>
@@ -4520,10 +4566,14 @@
         </is>
       </c>
       <c r="F6" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B6)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B6,'XTab DS_1'!$D$2:$D$106,$D6)</f>
         <v/>
       </c>
-      <c r="G6" s="11">
+      <c r="H6" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B6,'XTab DS_1'!$D$2:$D$106,$D6)</f>
         <v/>
       </c>
@@ -4555,10 +4605,14 @@
         </is>
       </c>
       <c r="F7" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B7)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G7" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B7,'XTab DS_1'!$D$2:$D$106,$D7)</f>
         <v/>
       </c>
-      <c r="G7" s="11">
+      <c r="H7" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B7,'XTab DS_1'!$D$2:$D$106,$D7)</f>
         <v/>
       </c>
@@ -4590,10 +4644,14 @@
         </is>
       </c>
       <c r="F8" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B8)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G8" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B8,'XTab DS_1'!$D$2:$D$106,$D8)</f>
         <v/>
       </c>
-      <c r="G8" s="11">
+      <c r="H8" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B8,'XTab DS_1'!$D$2:$D$106,$D8)</f>
         <v/>
       </c>
@@ -4625,10 +4683,14 @@
         </is>
       </c>
       <c r="F9" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B9)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G9" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B9,'XTab DS_1'!$D$2:$D$106,$D9)</f>
         <v/>
       </c>
-      <c r="G9" s="11">
+      <c r="H9" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B9,'XTab DS_1'!$D$2:$D$106,$D9)</f>
         <v/>
       </c>
@@ -4660,10 +4722,14 @@
         </is>
       </c>
       <c r="F10" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B10)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G10" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B10,'XTab DS_1'!$D$2:$D$106,$D10)</f>
         <v/>
       </c>
-      <c r="G10" s="11">
+      <c r="H10" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B10,'XTab DS_1'!$D$2:$D$106,$D10)</f>
         <v/>
       </c>
@@ -4695,10 +4761,14 @@
         </is>
       </c>
       <c r="F11" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B11)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G11" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B11,'XTab DS_1'!$D$2:$D$106,$D11)</f>
         <v/>
       </c>
-      <c r="G11" s="11">
+      <c r="H11" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B11,'XTab DS_1'!$D$2:$D$106,$D11)</f>
         <v/>
       </c>
@@ -4730,10 +4800,14 @@
         </is>
       </c>
       <c r="F12" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B12)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G12" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B12,'XTab DS_1'!$D$2:$D$106,$D12)</f>
         <v/>
       </c>
-      <c r="G12" s="11">
+      <c r="H12" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B12,'XTab DS_1'!$D$2:$D$106,$D12)</f>
         <v/>
       </c>
@@ -4765,10 +4839,14 @@
         </is>
       </c>
       <c r="F13" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B13)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G13" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B13,'XTab DS_1'!$D$2:$D$106,$D13)</f>
         <v/>
       </c>
-      <c r="G13" s="11">
+      <c r="H13" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B13,'XTab DS_1'!$D$2:$D$106,$D13)</f>
         <v/>
       </c>
@@ -4800,10 +4878,14 @@
         </is>
       </c>
       <c r="F14" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B14)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G14" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B14,'XTab DS_1'!$D$2:$D$106,$D14)</f>
         <v/>
       </c>
-      <c r="G14" s="11">
+      <c r="H14" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B14,'XTab DS_1'!$D$2:$D$106,$D14)</f>
         <v/>
       </c>
@@ -4835,10 +4917,14 @@
         </is>
       </c>
       <c r="F15" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B15)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G15" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B15,'XTab DS_1'!$D$2:$D$106,$D15)</f>
         <v/>
       </c>
-      <c r="G15" s="11">
+      <c r="H15" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B15,'XTab DS_1'!$D$2:$D$106,$D15)</f>
         <v/>
       </c>
@@ -4870,10 +4956,14 @@
         </is>
       </c>
       <c r="F16" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B16)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G16" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B16,'XTab DS_1'!$D$2:$D$106,$D16)</f>
         <v/>
       </c>
-      <c r="G16" s="11">
+      <c r="H16" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B16,'XTab DS_1'!$D$2:$D$106,$D16)</f>
         <v/>
       </c>
@@ -4905,10 +4995,14 @@
         </is>
       </c>
       <c r="F17" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B17)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G17" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B17,'XTab DS_1'!$D$2:$D$106,$D17)</f>
         <v/>
       </c>
-      <c r="G17" s="11">
+      <c r="H17" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B17,'XTab DS_1'!$D$2:$D$106,$D17)</f>
         <v/>
       </c>
@@ -4940,10 +5034,14 @@
         </is>
       </c>
       <c r="F18" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B18)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G18" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B18,'XTab DS_1'!$D$2:$D$106,$D18)</f>
         <v/>
       </c>
-      <c r="G18" s="11">
+      <c r="H18" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B18,'XTab DS_1'!$D$2:$D$106,$D18)</f>
         <v/>
       </c>
@@ -4975,10 +5073,14 @@
         </is>
       </c>
       <c r="F19" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B19)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G19" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B19,'XTab DS_1'!$D$2:$D$106,$D19)</f>
         <v/>
       </c>
-      <c r="G19" s="11">
+      <c r="H19" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B19,'XTab DS_1'!$D$2:$D$106,$D19)</f>
         <v/>
       </c>
@@ -5010,10 +5112,14 @@
         </is>
       </c>
       <c r="F20" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B20)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G20" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B20,'XTab DS_1'!$D$2:$D$106,$D20)</f>
         <v/>
       </c>
-      <c r="G20" s="11">
+      <c r="H20" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B20,'XTab DS_1'!$D$2:$D$106,$D20)</f>
         <v/>
       </c>
@@ -5045,10 +5151,14 @@
         </is>
       </c>
       <c r="F21" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B21)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G21" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B21,'XTab DS_1'!$D$2:$D$106,$D21)</f>
         <v/>
       </c>
-      <c r="G21" s="11">
+      <c r="H21" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B21,'XTab DS_1'!$D$2:$D$106,$D21)</f>
         <v/>
       </c>
@@ -5080,10 +5190,14 @@
         </is>
       </c>
       <c r="F22" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B22)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G22" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B22,'XTab DS_1'!$D$2:$D$106,$D22)</f>
         <v/>
       </c>
-      <c r="G22" s="11">
+      <c r="H22" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B22,'XTab DS_1'!$D$2:$D$106,$D22)</f>
         <v/>
       </c>
@@ -5115,10 +5229,14 @@
         </is>
       </c>
       <c r="F23" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B23)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G23" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B23,'XTab DS_1'!$D$2:$D$106,$D23)</f>
         <v/>
       </c>
-      <c r="G23" s="11">
+      <c r="H23" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B23,'XTab DS_1'!$D$2:$D$106,$D23)</f>
         <v/>
       </c>
@@ -5150,10 +5268,14 @@
         </is>
       </c>
       <c r="F24" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B24)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G24" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B24,'XTab DS_1'!$D$2:$D$106,$D24)</f>
         <v/>
       </c>
-      <c r="G24" s="11">
+      <c r="H24" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B24,'XTab DS_1'!$D$2:$D$106,$D24)</f>
         <v/>
       </c>
@@ -5185,10 +5307,14 @@
         </is>
       </c>
       <c r="F25" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B25)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G25" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B25,'XTab DS_1'!$D$2:$D$106,$D25)</f>
         <v/>
       </c>
-      <c r="G25" s="11">
+      <c r="H25" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B25,'XTab DS_1'!$D$2:$D$106,$D25)</f>
         <v/>
       </c>
@@ -5220,10 +5346,14 @@
         </is>
       </c>
       <c r="F26" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B26)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G26" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B26,'XTab DS_1'!$D$2:$D$106,$D26)</f>
         <v/>
       </c>
-      <c r="G26" s="11">
+      <c r="H26" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B26,'XTab DS_1'!$D$2:$D$106,$D26)</f>
         <v/>
       </c>
@@ -5255,10 +5385,14 @@
         </is>
       </c>
       <c r="F27" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B27)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G27" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B27,'XTab DS_1'!$D$2:$D$106,$D27)</f>
         <v/>
       </c>
-      <c r="G27" s="11">
+      <c r="H27" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B27,'XTab DS_1'!$D$2:$D$106,$D27)</f>
         <v/>
       </c>
@@ -5290,10 +5424,14 @@
         </is>
       </c>
       <c r="F28" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B28)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G28" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B28,'XTab DS_1'!$D$2:$D$106,$D28)</f>
         <v/>
       </c>
-      <c r="G28" s="11">
+      <c r="H28" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B28,'XTab DS_1'!$D$2:$D$106,$D28)</f>
         <v/>
       </c>
@@ -5325,10 +5463,14 @@
         </is>
       </c>
       <c r="F29" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B29)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G29" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B29,'XTab DS_1'!$D$2:$D$106,$D29)</f>
         <v/>
       </c>
-      <c r="G29" s="11">
+      <c r="H29" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B29,'XTab DS_1'!$D$2:$D$106,$D29)</f>
         <v/>
       </c>
@@ -5360,10 +5502,14 @@
         </is>
       </c>
       <c r="F30" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B30)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G30" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B30,'XTab DS_1'!$D$2:$D$106,$D30)</f>
         <v/>
       </c>
-      <c r="G30" s="11">
+      <c r="H30" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B30,'XTab DS_1'!$D$2:$D$106,$D30)</f>
         <v/>
       </c>
@@ -5395,10 +5541,14 @@
         </is>
       </c>
       <c r="F31" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B31)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G31" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B31,'XTab DS_1'!$D$2:$D$106,$D31)</f>
         <v/>
       </c>
-      <c r="G31" s="11">
+      <c r="H31" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B31,'XTab DS_1'!$D$2:$D$106,$D31)</f>
         <v/>
       </c>
@@ -5430,10 +5580,14 @@
         </is>
       </c>
       <c r="F32" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B32)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G32" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B32,'XTab DS_1'!$D$2:$D$106,$D32)</f>
         <v/>
       </c>
-      <c r="G32" s="11">
+      <c r="H32" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B32,'XTab DS_1'!$D$2:$D$106,$D32)</f>
         <v/>
       </c>
@@ -5465,10 +5619,14 @@
         </is>
       </c>
       <c r="F33" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B33)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G33" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B33,'XTab DS_1'!$D$2:$D$106,$D33)</f>
         <v/>
       </c>
-      <c r="G33" s="11">
+      <c r="H33" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B33,'XTab DS_1'!$D$2:$D$106,$D33)</f>
         <v/>
       </c>
@@ -5500,10 +5658,14 @@
         </is>
       </c>
       <c r="F34" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B34)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G34" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B34,'XTab DS_1'!$D$2:$D$106,$D34)</f>
         <v/>
       </c>
-      <c r="G34" s="11">
+      <c r="H34" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B34,'XTab DS_1'!$D$2:$D$106,$D34)</f>
         <v/>
       </c>
@@ -5535,10 +5697,14 @@
         </is>
       </c>
       <c r="F35" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B35)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G35" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B35,'XTab DS_1'!$D$2:$D$106,$D35)</f>
         <v/>
       </c>
-      <c r="G35" s="11">
+      <c r="H35" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B35,'XTab DS_1'!$D$2:$D$106,$D35)</f>
         <v/>
       </c>
@@ -5570,10 +5736,14 @@
         </is>
       </c>
       <c r="F36" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B36)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G36" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B36,'XTab DS_1'!$D$2:$D$106,$D36)</f>
         <v/>
       </c>
-      <c r="G36" s="11">
+      <c r="H36" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B36,'XTab DS_1'!$D$2:$D$106,$D36)</f>
         <v/>
       </c>
@@ -5605,10 +5775,14 @@
         </is>
       </c>
       <c r="F37" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B37)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G37" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B37,'XTab DS_1'!$D$2:$D$106,$D37)</f>
         <v/>
       </c>
-      <c r="G37" s="11">
+      <c r="H37" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B37,'XTab DS_1'!$D$2:$D$106,$D37)</f>
         <v/>
       </c>
@@ -5640,10 +5814,14 @@
         </is>
       </c>
       <c r="F38" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B38)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G38" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B38,'XTab DS_1'!$D$2:$D$106,$D38)</f>
         <v/>
       </c>
-      <c r="G38" s="11">
+      <c r="H38" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B38,'XTab DS_1'!$D$2:$D$106,$D38)</f>
         <v/>
       </c>
@@ -5675,10 +5853,14 @@
         </is>
       </c>
       <c r="F39" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B39)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G39" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B39,'XTab DS_1'!$D$2:$D$106,$D39)</f>
         <v/>
       </c>
-      <c r="G39" s="11">
+      <c r="H39" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B39,'XTab DS_1'!$D$2:$D$106,$D39)</f>
         <v/>
       </c>
@@ -5710,10 +5892,14 @@
         </is>
       </c>
       <c r="F40" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B40)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G40" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B40,'XTab DS_1'!$D$2:$D$106,$D40)</f>
         <v/>
       </c>
-      <c r="G40" s="11">
+      <c r="H40" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B40,'XTab DS_1'!$D$2:$D$106,$D40)</f>
         <v/>
       </c>
@@ -5745,10 +5931,14 @@
         </is>
       </c>
       <c r="F41" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B41)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G41" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B41,'XTab DS_1'!$D$2:$D$106,$D41)</f>
         <v/>
       </c>
-      <c r="G41" s="11">
+      <c r="H41" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B41,'XTab DS_1'!$D$2:$D$106,$D41)</f>
         <v/>
       </c>
@@ -5780,10 +5970,14 @@
         </is>
       </c>
       <c r="F42" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B42)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G42" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B42,'XTab DS_1'!$D$2:$D$106,$D42)</f>
         <v/>
       </c>
-      <c r="G42" s="11">
+      <c r="H42" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B42,'XTab DS_1'!$D$2:$D$106,$D42)</f>
         <v/>
       </c>
@@ -5815,10 +6009,14 @@
         </is>
       </c>
       <c r="F43" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B43)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G43" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B43,'XTab DS_1'!$D$2:$D$106,$D43)</f>
         <v/>
       </c>
-      <c r="G43" s="11">
+      <c r="H43" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B43,'XTab DS_1'!$D$2:$D$106,$D43)</f>
         <v/>
       </c>
@@ -5850,10 +6048,14 @@
         </is>
       </c>
       <c r="F44" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B44)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G44" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B44,'XTab DS_1'!$D$2:$D$106,$D44)</f>
         <v/>
       </c>
-      <c r="G44" s="11">
+      <c r="H44" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B44,'XTab DS_1'!$D$2:$D$106,$D44)</f>
         <v/>
       </c>
@@ -5885,10 +6087,14 @@
         </is>
       </c>
       <c r="F45" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B45)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G45" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B45,'XTab DS_1'!$D$2:$D$106,$D45)</f>
         <v/>
       </c>
-      <c r="G45" s="11">
+      <c r="H45" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B45,'XTab DS_1'!$D$2:$D$106,$D45)</f>
         <v/>
       </c>
@@ -5920,10 +6126,14 @@
         </is>
       </c>
       <c r="F46" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B46)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G46" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B46,'XTab DS_1'!$D$2:$D$106,$D46)</f>
         <v/>
       </c>
-      <c r="G46" s="11">
+      <c r="H46" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B46,'XTab DS_1'!$D$2:$D$106,$D46)</f>
         <v/>
       </c>
@@ -5955,10 +6165,14 @@
         </is>
       </c>
       <c r="F47" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B47)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G47" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B47,'XTab DS_1'!$D$2:$D$106,$D47)</f>
         <v/>
       </c>
-      <c r="G47" s="11">
+      <c r="H47" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B47,'XTab DS_1'!$D$2:$D$106,$D47)</f>
         <v/>
       </c>
@@ -5990,10 +6204,14 @@
         </is>
       </c>
       <c r="F48" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B48)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G48" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B48,'XTab DS_1'!$D$2:$D$106,$D48)</f>
         <v/>
       </c>
-      <c r="G48" s="11">
+      <c r="H48" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B48,'XTab DS_1'!$D$2:$D$106,$D48)</f>
         <v/>
       </c>
@@ -6025,10 +6243,14 @@
         </is>
       </c>
       <c r="F49" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B49)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G49" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B49,'XTab DS_1'!$D$2:$D$106,$D49)</f>
         <v/>
       </c>
-      <c r="G49" s="11">
+      <c r="H49" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B49,'XTab DS_1'!$D$2:$D$106,$D49)</f>
         <v/>
       </c>
@@ -6060,10 +6282,14 @@
         </is>
       </c>
       <c r="F50" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B50)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G50" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B50,'XTab DS_1'!$D$2:$D$106,$D50)</f>
         <v/>
       </c>
-      <c r="G50" s="11">
+      <c r="H50" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B50,'XTab DS_1'!$D$2:$D$106,$D50)</f>
         <v/>
       </c>
@@ -6095,10 +6321,14 @@
         </is>
       </c>
       <c r="F51" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B51)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G51" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B51,'XTab DS_1'!$D$2:$D$106,$D51)</f>
         <v/>
       </c>
-      <c r="G51" s="11">
+      <c r="H51" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B51,'XTab DS_1'!$D$2:$D$106,$D51)</f>
         <v/>
       </c>
@@ -6130,10 +6360,14 @@
         </is>
       </c>
       <c r="F52" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B52)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G52" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B52,'XTab DS_1'!$D$2:$D$106,$D52)</f>
         <v/>
       </c>
-      <c r="G52" s="11">
+      <c r="H52" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B52,'XTab DS_1'!$D$2:$D$106,$D52)</f>
         <v/>
       </c>
@@ -6165,35 +6399,119 @@
         </is>
       </c>
       <c r="F53" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B53)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G53" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B53,'XTab DS_1'!$D$2:$D$106,$D53)</f>
         <v/>
       </c>
-      <c r="G53" s="11">
+      <c r="H53" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B53,'XTab DS_1'!$D$2:$D$106,$D53)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n"/>
-      <c r="B54" s="12" t="n"/>
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>QCX2412FRNPTFN-10</t>
+        </is>
+      </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
+          <t>葬送のフリーレンP 経費（課税10％）</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>CX01</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="inlineStr">
+        <is>
+          <t>CX催事</t>
+        </is>
+      </c>
+      <c r="F54" s="14">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B54)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G54" s="15">
+        <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B54,'XTab DS_1'!$D$2:$D$106,$D54)</f>
+        <v/>
+      </c>
+      <c r="H54" s="16">
+        <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B54,'XTab DS_1'!$D$2:$D$106,$D54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="17" t="n"/>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D54" s="12" t="n"/>
-      <c r="E54" s="12" t="n"/>
-      <c r="F54" s="14">
-        <f>SUM(F2:F53)</f>
-        <v/>
-      </c>
-      <c r="G54" s="15">
-        <f>SUM(G2:G53)</f>
+      <c r="D55" s="17" t="n"/>
+      <c r="E55" s="17" t="n"/>
+      <c r="F55" s="17" t="n"/>
+      <c r="G55" s="19">
+        <f>SUM(G2:G54)</f>
+        <v/>
+      </c>
+      <c r="H55" s="20">
+        <f>SUM(H2:H54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="21" t="n"/>
+      <c r="B56" s="21" t="n"/>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>うち 重複</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="n"/>
+      <c r="E56" s="21" t="n"/>
+      <c r="F56" s="21" t="n"/>
+      <c r="G56" s="23">
+        <f>SUMIFS(G2:G54,F2:F54,"重複")</f>
+        <v/>
+      </c>
+      <c r="H56" s="24">
+        <f>SUMIFS(H2:H54,F2:F54,"重複")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="21" t="n"/>
+      <c r="B57" s="21" t="n"/>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>うち 単独</t>
+        </is>
+      </c>
+      <c r="D57" s="21" t="n"/>
+      <c r="E57" s="21" t="n"/>
+      <c r="F57" s="21" t="n"/>
+      <c r="G57" s="23">
+        <f>SUMIFS(G2:G54,F2:F54,"単独")</f>
+        <v/>
+      </c>
+      <c r="H57" s="24">
+        <f>SUMIFS(H2:H54,F2:F54,"単独")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6204,7 +6522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="2" min="1" max="1"/>
@@ -6212,8 +6530,9 @@
     <col width="52" customWidth="1" style="2" min="3" max="3"/>
     <col width="10" customWidth="1" style="2" min="4" max="4"/>
     <col width="12" customWidth="1" style="2" min="5" max="5"/>
-    <col width="14" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
+    <col width="8" customWidth="1" style="2" min="6" max="6"/>
+    <col width="14" customWidth="1" style="2" min="7" max="7"/>
+    <col width="16" customWidth="1" style="2" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6244,10 +6563,15 @@
       </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
           <t>在庫数量</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>在庫金額</t>
         </is>
@@ -6280,10 +6604,14 @@
         </is>
       </c>
       <c r="F2" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B2)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G2" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B2,'XTab DS_1'!$D$2:$D$106,$D2)</f>
         <v/>
       </c>
-      <c r="G2" s="11">
+      <c r="H2" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B2,'XTab DS_1'!$D$2:$D$106,$D2)</f>
         <v/>
       </c>
@@ -6315,10 +6643,14 @@
         </is>
       </c>
       <c r="F3" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B3)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G3" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B3,'XTab DS_1'!$D$2:$D$106,$D3)</f>
         <v/>
       </c>
-      <c r="G3" s="11">
+      <c r="H3" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B3,'XTab DS_1'!$D$2:$D$106,$D3)</f>
         <v/>
       </c>
@@ -6350,10 +6682,14 @@
         </is>
       </c>
       <c r="F4" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B4)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G4" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B4,'XTab DS_1'!$D$2:$D$106,$D4)</f>
         <v/>
       </c>
-      <c r="G4" s="11">
+      <c r="H4" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B4,'XTab DS_1'!$D$2:$D$106,$D4)</f>
         <v/>
       </c>
@@ -6385,10 +6721,14 @@
         </is>
       </c>
       <c r="F5" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B5)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G5" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B5,'XTab DS_1'!$D$2:$D$106,$D5)</f>
         <v/>
       </c>
-      <c r="G5" s="11">
+      <c r="H5" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B5,'XTab DS_1'!$D$2:$D$106,$D5)</f>
         <v/>
       </c>
@@ -6420,10 +6760,14 @@
         </is>
       </c>
       <c r="F6" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B6)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B6,'XTab DS_1'!$D$2:$D$106,$D6)</f>
         <v/>
       </c>
-      <c r="G6" s="11">
+      <c r="H6" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B6,'XTab DS_1'!$D$2:$D$106,$D6)</f>
         <v/>
       </c>
@@ -6455,10 +6799,14 @@
         </is>
       </c>
       <c r="F7" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B7)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G7" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B7,'XTab DS_1'!$D$2:$D$106,$D7)</f>
         <v/>
       </c>
-      <c r="G7" s="11">
+      <c r="H7" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B7,'XTab DS_1'!$D$2:$D$106,$D7)</f>
         <v/>
       </c>
@@ -6490,10 +6838,14 @@
         </is>
       </c>
       <c r="F8" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B8)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G8" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B8,'XTab DS_1'!$D$2:$D$106,$D8)</f>
         <v/>
       </c>
-      <c r="G8" s="11">
+      <c r="H8" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B8,'XTab DS_1'!$D$2:$D$106,$D8)</f>
         <v/>
       </c>
@@ -6525,10 +6877,14 @@
         </is>
       </c>
       <c r="F9" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B9)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G9" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B9,'XTab DS_1'!$D$2:$D$106,$D9)</f>
         <v/>
       </c>
-      <c r="G9" s="11">
+      <c r="H9" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B9,'XTab DS_1'!$D$2:$D$106,$D9)</f>
         <v/>
       </c>
@@ -6560,10 +6916,14 @@
         </is>
       </c>
       <c r="F10" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B10)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G10" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B10,'XTab DS_1'!$D$2:$D$106,$D10)</f>
         <v/>
       </c>
-      <c r="G10" s="11">
+      <c r="H10" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B10,'XTab DS_1'!$D$2:$D$106,$D10)</f>
         <v/>
       </c>
@@ -6595,10 +6955,14 @@
         </is>
       </c>
       <c r="F11" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B11)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G11" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B11,'XTab DS_1'!$D$2:$D$106,$D11)</f>
         <v/>
       </c>
-      <c r="G11" s="11">
+      <c r="H11" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B11,'XTab DS_1'!$D$2:$D$106,$D11)</f>
         <v/>
       </c>
@@ -6630,10 +6994,14 @@
         </is>
       </c>
       <c r="F12" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B12)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G12" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B12,'XTab DS_1'!$D$2:$D$106,$D12)</f>
         <v/>
       </c>
-      <c r="G12" s="11">
+      <c r="H12" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B12,'XTab DS_1'!$D$2:$D$106,$D12)</f>
         <v/>
       </c>
@@ -6665,10 +7033,14 @@
         </is>
       </c>
       <c r="F13" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B13)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G13" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B13,'XTab DS_1'!$D$2:$D$106,$D13)</f>
         <v/>
       </c>
-      <c r="G13" s="11">
+      <c r="H13" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B13,'XTab DS_1'!$D$2:$D$106,$D13)</f>
         <v/>
       </c>
@@ -6700,10 +7072,14 @@
         </is>
       </c>
       <c r="F14" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B14)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G14" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B14,'XTab DS_1'!$D$2:$D$106,$D14)</f>
         <v/>
       </c>
-      <c r="G14" s="11">
+      <c r="H14" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B14,'XTab DS_1'!$D$2:$D$106,$D14)</f>
         <v/>
       </c>
@@ -6735,10 +7111,14 @@
         </is>
       </c>
       <c r="F15" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B15)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G15" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B15,'XTab DS_1'!$D$2:$D$106,$D15)</f>
         <v/>
       </c>
-      <c r="G15" s="11">
+      <c r="H15" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B15,'XTab DS_1'!$D$2:$D$106,$D15)</f>
         <v/>
       </c>
@@ -6770,10 +7150,14 @@
         </is>
       </c>
       <c r="F16" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B16)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G16" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B16,'XTab DS_1'!$D$2:$D$106,$D16)</f>
         <v/>
       </c>
-      <c r="G16" s="11">
+      <c r="H16" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B16,'XTab DS_1'!$D$2:$D$106,$D16)</f>
         <v/>
       </c>
@@ -6805,10 +7189,14 @@
         </is>
       </c>
       <c r="F17" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B17)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G17" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B17,'XTab DS_1'!$D$2:$D$106,$D17)</f>
         <v/>
       </c>
-      <c r="G17" s="11">
+      <c r="H17" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B17,'XTab DS_1'!$D$2:$D$106,$D17)</f>
         <v/>
       </c>
@@ -6840,10 +7228,14 @@
         </is>
       </c>
       <c r="F18" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B18)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G18" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B18,'XTab DS_1'!$D$2:$D$106,$D18)</f>
         <v/>
       </c>
-      <c r="G18" s="11">
+      <c r="H18" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B18,'XTab DS_1'!$D$2:$D$106,$D18)</f>
         <v/>
       </c>
@@ -6875,10 +7267,14 @@
         </is>
       </c>
       <c r="F19" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B19)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G19" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B19,'XTab DS_1'!$D$2:$D$106,$D19)</f>
         <v/>
       </c>
-      <c r="G19" s="11">
+      <c r="H19" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B19,'XTab DS_1'!$D$2:$D$106,$D19)</f>
         <v/>
       </c>
@@ -6910,10 +7306,14 @@
         </is>
       </c>
       <c r="F20" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B20)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G20" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B20,'XTab DS_1'!$D$2:$D$106,$D20)</f>
         <v/>
       </c>
-      <c r="G20" s="11">
+      <c r="H20" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B20,'XTab DS_1'!$D$2:$D$106,$D20)</f>
         <v/>
       </c>
@@ -6945,10 +7345,14 @@
         </is>
       </c>
       <c r="F21" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B21)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G21" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B21,'XTab DS_1'!$D$2:$D$106,$D21)</f>
         <v/>
       </c>
-      <c r="G21" s="11">
+      <c r="H21" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B21,'XTab DS_1'!$D$2:$D$106,$D21)</f>
         <v/>
       </c>
@@ -6980,10 +7384,14 @@
         </is>
       </c>
       <c r="F22" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B22)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G22" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B22,'XTab DS_1'!$D$2:$D$106,$D22)</f>
         <v/>
       </c>
-      <c r="G22" s="11">
+      <c r="H22" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B22,'XTab DS_1'!$D$2:$D$106,$D22)</f>
         <v/>
       </c>
@@ -7015,10 +7423,14 @@
         </is>
       </c>
       <c r="F23" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B23)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G23" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B23,'XTab DS_1'!$D$2:$D$106,$D23)</f>
         <v/>
       </c>
-      <c r="G23" s="11">
+      <c r="H23" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B23,'XTab DS_1'!$D$2:$D$106,$D23)</f>
         <v/>
       </c>
@@ -7050,10 +7462,14 @@
         </is>
       </c>
       <c r="F24" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B24)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G24" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B24,'XTab DS_1'!$D$2:$D$106,$D24)</f>
         <v/>
       </c>
-      <c r="G24" s="11">
+      <c r="H24" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B24,'XTab DS_1'!$D$2:$D$106,$D24)</f>
         <v/>
       </c>
@@ -7085,10 +7501,14 @@
         </is>
       </c>
       <c r="F25" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B25)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G25" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B25,'XTab DS_1'!$D$2:$D$106,$D25)</f>
         <v/>
       </c>
-      <c r="G25" s="11">
+      <c r="H25" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B25,'XTab DS_1'!$D$2:$D$106,$D25)</f>
         <v/>
       </c>
@@ -7120,10 +7540,14 @@
         </is>
       </c>
       <c r="F26" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B26)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G26" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B26,'XTab DS_1'!$D$2:$D$106,$D26)</f>
         <v/>
       </c>
-      <c r="G26" s="11">
+      <c r="H26" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B26,'XTab DS_1'!$D$2:$D$106,$D26)</f>
         <v/>
       </c>
@@ -7155,10 +7579,14 @@
         </is>
       </c>
       <c r="F27" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B27)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G27" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B27,'XTab DS_1'!$D$2:$D$106,$D27)</f>
         <v/>
       </c>
-      <c r="G27" s="11">
+      <c r="H27" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B27,'XTab DS_1'!$D$2:$D$106,$D27)</f>
         <v/>
       </c>
@@ -7190,10 +7618,14 @@
         </is>
       </c>
       <c r="F28" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B28)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G28" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B28,'XTab DS_1'!$D$2:$D$106,$D28)</f>
         <v/>
       </c>
-      <c r="G28" s="11">
+      <c r="H28" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B28,'XTab DS_1'!$D$2:$D$106,$D28)</f>
         <v/>
       </c>
@@ -7225,10 +7657,14 @@
         </is>
       </c>
       <c r="F29" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B29)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G29" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B29,'XTab DS_1'!$D$2:$D$106,$D29)</f>
         <v/>
       </c>
-      <c r="G29" s="11">
+      <c r="H29" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B29,'XTab DS_1'!$D$2:$D$106,$D29)</f>
         <v/>
       </c>
@@ -7260,10 +7696,14 @@
         </is>
       </c>
       <c r="F30" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B30)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G30" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B30,'XTab DS_1'!$D$2:$D$106,$D30)</f>
         <v/>
       </c>
-      <c r="G30" s="11">
+      <c r="H30" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B30,'XTab DS_1'!$D$2:$D$106,$D30)</f>
         <v/>
       </c>
@@ -7295,10 +7735,14 @@
         </is>
       </c>
       <c r="F31" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B31)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G31" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B31,'XTab DS_1'!$D$2:$D$106,$D31)</f>
         <v/>
       </c>
-      <c r="G31" s="11">
+      <c r="H31" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B31,'XTab DS_1'!$D$2:$D$106,$D31)</f>
         <v/>
       </c>
@@ -7330,10 +7774,14 @@
         </is>
       </c>
       <c r="F32" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B32)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G32" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B32,'XTab DS_1'!$D$2:$D$106,$D32)</f>
         <v/>
       </c>
-      <c r="G32" s="11">
+      <c r="H32" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B32,'XTab DS_1'!$D$2:$D$106,$D32)</f>
         <v/>
       </c>
@@ -7365,10 +7813,14 @@
         </is>
       </c>
       <c r="F33" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B33)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G33" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B33,'XTab DS_1'!$D$2:$D$106,$D33)</f>
         <v/>
       </c>
-      <c r="G33" s="11">
+      <c r="H33" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B33,'XTab DS_1'!$D$2:$D$106,$D33)</f>
         <v/>
       </c>
@@ -7400,10 +7852,14 @@
         </is>
       </c>
       <c r="F34" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B34)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G34" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B34,'XTab DS_1'!$D$2:$D$106,$D34)</f>
         <v/>
       </c>
-      <c r="G34" s="11">
+      <c r="H34" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B34,'XTab DS_1'!$D$2:$D$106,$D34)</f>
         <v/>
       </c>
@@ -7435,10 +7891,14 @@
         </is>
       </c>
       <c r="F35" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B35)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G35" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B35,'XTab DS_1'!$D$2:$D$106,$D35)</f>
         <v/>
       </c>
-      <c r="G35" s="11">
+      <c r="H35" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B35,'XTab DS_1'!$D$2:$D$106,$D35)</f>
         <v/>
       </c>
@@ -7470,10 +7930,14 @@
         </is>
       </c>
       <c r="F36" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B36)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G36" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B36,'XTab DS_1'!$D$2:$D$106,$D36)</f>
         <v/>
       </c>
-      <c r="G36" s="11">
+      <c r="H36" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B36,'XTab DS_1'!$D$2:$D$106,$D36)</f>
         <v/>
       </c>
@@ -7505,10 +7969,14 @@
         </is>
       </c>
       <c r="F37" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B37)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G37" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B37,'XTab DS_1'!$D$2:$D$106,$D37)</f>
         <v/>
       </c>
-      <c r="G37" s="11">
+      <c r="H37" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B37,'XTab DS_1'!$D$2:$D$106,$D37)</f>
         <v/>
       </c>
@@ -7540,10 +8008,14 @@
         </is>
       </c>
       <c r="F38" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B38)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G38" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B38,'XTab DS_1'!$D$2:$D$106,$D38)</f>
         <v/>
       </c>
-      <c r="G38" s="11">
+      <c r="H38" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B38,'XTab DS_1'!$D$2:$D$106,$D38)</f>
         <v/>
       </c>
@@ -7575,10 +8047,14 @@
         </is>
       </c>
       <c r="F39" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B39)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G39" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B39,'XTab DS_1'!$D$2:$D$106,$D39)</f>
         <v/>
       </c>
-      <c r="G39" s="11">
+      <c r="H39" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B39,'XTab DS_1'!$D$2:$D$106,$D39)</f>
         <v/>
       </c>
@@ -7610,10 +8086,14 @@
         </is>
       </c>
       <c r="F40" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B40)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G40" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B40,'XTab DS_1'!$D$2:$D$106,$D40)</f>
         <v/>
       </c>
-      <c r="G40" s="11">
+      <c r="H40" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B40,'XTab DS_1'!$D$2:$D$106,$D40)</f>
         <v/>
       </c>
@@ -7645,10 +8125,14 @@
         </is>
       </c>
       <c r="F41" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B41)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G41" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B41,'XTab DS_1'!$D$2:$D$106,$D41)</f>
         <v/>
       </c>
-      <c r="G41" s="11">
+      <c r="H41" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B41,'XTab DS_1'!$D$2:$D$106,$D41)</f>
         <v/>
       </c>
@@ -7680,10 +8164,14 @@
         </is>
       </c>
       <c r="F42" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B42)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G42" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B42,'XTab DS_1'!$D$2:$D$106,$D42)</f>
         <v/>
       </c>
-      <c r="G42" s="11">
+      <c r="H42" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B42,'XTab DS_1'!$D$2:$D$106,$D42)</f>
         <v/>
       </c>
@@ -7715,10 +8203,14 @@
         </is>
       </c>
       <c r="F43" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B43)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G43" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B43,'XTab DS_1'!$D$2:$D$106,$D43)</f>
         <v/>
       </c>
-      <c r="G43" s="11">
+      <c r="H43" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B43,'XTab DS_1'!$D$2:$D$106,$D43)</f>
         <v/>
       </c>
@@ -7750,10 +8242,14 @@
         </is>
       </c>
       <c r="F44" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B44)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G44" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B44,'XTab DS_1'!$D$2:$D$106,$D44)</f>
         <v/>
       </c>
-      <c r="G44" s="11">
+      <c r="H44" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B44,'XTab DS_1'!$D$2:$D$106,$D44)</f>
         <v/>
       </c>
@@ -7785,10 +8281,14 @@
         </is>
       </c>
       <c r="F45" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B45)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G45" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B45,'XTab DS_1'!$D$2:$D$106,$D45)</f>
         <v/>
       </c>
-      <c r="G45" s="11">
+      <c r="H45" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B45,'XTab DS_1'!$D$2:$D$106,$D45)</f>
         <v/>
       </c>
@@ -7820,10 +8320,14 @@
         </is>
       </c>
       <c r="F46" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B46)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G46" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B46,'XTab DS_1'!$D$2:$D$106,$D46)</f>
         <v/>
       </c>
-      <c r="G46" s="11">
+      <c r="H46" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B46,'XTab DS_1'!$D$2:$D$106,$D46)</f>
         <v/>
       </c>
@@ -7855,10 +8359,14 @@
         </is>
       </c>
       <c r="F47" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B47)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G47" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B47,'XTab DS_1'!$D$2:$D$106,$D47)</f>
         <v/>
       </c>
-      <c r="G47" s="11">
+      <c r="H47" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B47,'XTab DS_1'!$D$2:$D$106,$D47)</f>
         <v/>
       </c>
@@ -7890,10 +8398,14 @@
         </is>
       </c>
       <c r="F48" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B48)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G48" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B48,'XTab DS_1'!$D$2:$D$106,$D48)</f>
         <v/>
       </c>
-      <c r="G48" s="11">
+      <c r="H48" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B48,'XTab DS_1'!$D$2:$D$106,$D48)</f>
         <v/>
       </c>
@@ -7925,10 +8437,14 @@
         </is>
       </c>
       <c r="F49" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B49)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G49" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B49,'XTab DS_1'!$D$2:$D$106,$D49)</f>
         <v/>
       </c>
-      <c r="G49" s="11">
+      <c r="H49" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B49,'XTab DS_1'!$D$2:$D$106,$D49)</f>
         <v/>
       </c>
@@ -7960,10 +8476,14 @@
         </is>
       </c>
       <c r="F50" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B50)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G50" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B50,'XTab DS_1'!$D$2:$D$106,$D50)</f>
         <v/>
       </c>
-      <c r="G50" s="11">
+      <c r="H50" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B50,'XTab DS_1'!$D$2:$D$106,$D50)</f>
         <v/>
       </c>
@@ -7995,10 +8515,14 @@
         </is>
       </c>
       <c r="F51" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B51)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G51" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B51,'XTab DS_1'!$D$2:$D$106,$D51)</f>
         <v/>
       </c>
-      <c r="G51" s="11">
+      <c r="H51" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B51,'XTab DS_1'!$D$2:$D$106,$D51)</f>
         <v/>
       </c>
@@ -8030,10 +8554,14 @@
         </is>
       </c>
       <c r="F52" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B52)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G52" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B52,'XTab DS_1'!$D$2:$D$106,$D52)</f>
         <v/>
       </c>
-      <c r="G52" s="11">
+      <c r="H52" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B52,'XTab DS_1'!$D$2:$D$106,$D52)</f>
         <v/>
       </c>
@@ -8065,35 +8593,80 @@
         </is>
       </c>
       <c r="F53" s="10">
+        <f>IF(COUNTIFS('XTab DS_1'!$B$2:$B$106,$B53)&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="G53" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B53,'XTab DS_1'!$D$2:$D$106,$D53)</f>
         <v/>
       </c>
-      <c r="G53" s="11">
+      <c r="H53" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B53,'XTab DS_1'!$D$2:$D$106,$D53)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n"/>
-      <c r="B54" s="12" t="n"/>
-      <c r="C54" s="13" t="inlineStr">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="17" t="n"/>
+      <c r="C54" s="18" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D54" s="12" t="n"/>
-      <c r="E54" s="12" t="n"/>
-      <c r="F54" s="14">
-        <f>SUM(F2:F53)</f>
-        <v/>
-      </c>
-      <c r="G54" s="15">
+      <c r="D54" s="17" t="n"/>
+      <c r="E54" s="17" t="n"/>
+      <c r="F54" s="17" t="n"/>
+      <c r="G54" s="19">
         <f>SUM(G2:G53)</f>
         <v/>
       </c>
+      <c r="H54" s="20">
+        <f>SUM(H2:H53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="21" t="n"/>
+      <c r="B55" s="21" t="n"/>
+      <c r="C55" s="22" t="inlineStr">
+        <is>
+          <t>うち 重複</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="n"/>
+      <c r="E55" s="21" t="n"/>
+      <c r="F55" s="21" t="n"/>
+      <c r="G55" s="23">
+        <f>SUMIFS(G2:G53,F2:F53,"重複")</f>
+        <v/>
+      </c>
+      <c r="H55" s="24">
+        <f>SUMIFS(H2:H53,F2:F53,"重複")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="21" t="n"/>
+      <c r="B56" s="21" t="n"/>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>うち 単独</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="n"/>
+      <c r="E56" s="21" t="n"/>
+      <c r="F56" s="21" t="n"/>
+      <c r="G56" s="23">
+        <f>SUMIFS(G2:G53,F2:F53,"単独")</f>
+        <v/>
+      </c>
+      <c r="H56" s="24">
+        <f>SUMIFS(H2:H53,F2:F53,"単独")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8104,19 +8677,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="2" min="1" max="1"/>
     <col width="24" customWidth="1" style="2" min="2" max="2"/>
     <col width="52" customWidth="1" style="2" min="3" max="3"/>
     <col width="10" customWidth="1" style="2" min="4" max="4"/>
-    <col width="13" customWidth="1" style="2" min="5" max="5"/>
-    <col width="14" customWidth="1" style="2" min="6" max="6"/>
-    <col width="13" customWidth="1" style="2" min="7" max="7"/>
-    <col width="14" customWidth="1" style="2" min="8" max="8"/>
-    <col width="15" customWidth="1" style="2" min="9" max="9"/>
-    <col width="18" customWidth="1" style="2" min="10" max="10"/>
+    <col width="8" customWidth="1" style="2" min="5" max="5"/>
+    <col width="13" customWidth="1" style="2" min="6" max="6"/>
+    <col width="14" customWidth="1" style="2" min="7" max="7"/>
+    <col width="13" customWidth="1" style="2" min="8" max="8"/>
+    <col width="14" customWidth="1" style="2" min="9" max="9"/>
+    <col width="15" customWidth="1" style="2" min="10" max="10"/>
+    <col width="18" customWidth="1" style="2" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8137,35 +8711,40 @@
       </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
-          <t>重複倉庫数</t>
+          <t>登録倉庫数</t>
         </is>
       </c>
       <c r="E1" s="8" t="inlineStr">
         <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
           <t>CX催事 数量</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>CX催事 金額</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>DBS倉庫 数量</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>DBS倉庫 金額</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>合算 在庫数量</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>合算 在庫金額(原価)</t>
         </is>
@@ -8187,31 +8766,35 @@
           <t>葬送のフリーレンP　原画ランダム缶バッジ　全23種</t>
         </is>
       </c>
-      <c r="D2" s="16">
+      <c r="D2" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B2)</f>
         <v/>
       </c>
       <c r="E2" s="10">
+        <f>IF(D2&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F2" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B2,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F2" s="11">
+      <c r="G2" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B2,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G2" s="10">
+      <c r="H2" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B2,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H2" s="11">
+      <c r="I2" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B2,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I2" s="17">
+      <c r="J2" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B2)</f>
         <v/>
       </c>
-      <c r="J2" s="18">
+      <c r="K2" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B2)</f>
         <v/>
       </c>
@@ -8232,31 +8815,35 @@
           <t>葬送のフリーレンP　原画ランダムアクリルキーホルダー　全20種</t>
         </is>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B3)</f>
         <v/>
       </c>
       <c r="E3" s="10">
+        <f>IF(D3&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F3" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B3,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F3" s="11">
+      <c r="G3" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B3,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G3" s="10">
+      <c r="H3" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B3,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H3" s="11">
+      <c r="I3" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B3,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I3" s="17">
+      <c r="J3" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B3)</f>
         <v/>
       </c>
-      <c r="J3" s="18">
+      <c r="K3" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B3)</f>
         <v/>
       </c>
@@ -8277,31 +8864,35 @@
           <t>葬送のフリーレンP　A4クリアファイル　(フリーレン)</t>
         </is>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B4)</f>
         <v/>
       </c>
       <c r="E4" s="10">
+        <f>IF(D4&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F4" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B4,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F4" s="11">
+      <c r="G4" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B4,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G4" s="10">
+      <c r="H4" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B4,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H4" s="11">
+      <c r="I4" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B4,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I4" s="17">
+      <c r="J4" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B4)</f>
         <v/>
       </c>
-      <c r="J4" s="18">
+      <c r="K4" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B4)</f>
         <v/>
       </c>
@@ -8322,31 +8913,35 @@
           <t>葬送のフリーレンP　A4クリアファイル　(フェルン)</t>
         </is>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B5)</f>
         <v/>
       </c>
       <c r="E5" s="10">
+        <f>IF(D5&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F5" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B5,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F5" s="11">
+      <c r="G5" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B5,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G5" s="10">
+      <c r="H5" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B5,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H5" s="11">
+      <c r="I5" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B5,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I5" s="17">
+      <c r="J5" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B5)</f>
         <v/>
       </c>
-      <c r="J5" s="18">
+      <c r="K5" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B5)</f>
         <v/>
       </c>
@@ -8367,31 +8962,35 @@
           <t>葬送のフリーレンP　A4クリアファイル　(シュタルク)</t>
         </is>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B6)</f>
         <v/>
       </c>
       <c r="E6" s="10">
+        <f>IF(D6&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B6,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F6" s="11">
+      <c r="G6" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B6,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G6" s="10">
+      <c r="H6" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B6,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H6" s="11">
+      <c r="I6" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B6,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I6" s="17">
+      <c r="J6" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B6)</f>
         <v/>
       </c>
-      <c r="J6" s="18">
+      <c r="K6" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B6)</f>
         <v/>
       </c>
@@ -8412,31 +9011,35 @@
           <t>葬送のフリーレンP　アクリルスタンド　(フリーレン)</t>
         </is>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B7)</f>
         <v/>
       </c>
       <c r="E7" s="10">
+        <f>IF(D7&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F7" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B7,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F7" s="11">
+      <c r="G7" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B7,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G7" s="10">
+      <c r="H7" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B7,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H7" s="11">
+      <c r="I7" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B7,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I7" s="17">
+      <c r="J7" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B7)</f>
         <v/>
       </c>
-      <c r="J7" s="18">
+      <c r="K7" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B7)</f>
         <v/>
       </c>
@@ -8457,31 +9060,35 @@
           <t>葬送のフリーレンP　アクリルスタンド　(フェルン)</t>
         </is>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B8)</f>
         <v/>
       </c>
       <c r="E8" s="10">
+        <f>IF(D8&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F8" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B8,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F8" s="11">
+      <c r="G8" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B8,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G8" s="10">
+      <c r="H8" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B8,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H8" s="11">
+      <c r="I8" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B8,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I8" s="17">
+      <c r="J8" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B8)</f>
         <v/>
       </c>
-      <c r="J8" s="18">
+      <c r="K8" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B8)</f>
         <v/>
       </c>
@@ -8502,31 +9109,35 @@
           <t>葬送のフリーレンP　アクリルスタンド　(シュタルク)</t>
         </is>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B9)</f>
         <v/>
       </c>
       <c r="E9" s="10">
+        <f>IF(D9&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F9" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B9,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F9" s="11">
+      <c r="G9" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B9,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G9" s="10">
+      <c r="H9" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B9,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H9" s="11">
+      <c r="I9" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B9,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I9" s="17">
+      <c r="J9" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B9)</f>
         <v/>
       </c>
-      <c r="J9" s="18">
+      <c r="K9" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B9)</f>
         <v/>
       </c>
@@ -8547,31 +9158,35 @@
           <t>葬送のフリーレンP　缶バッジ　(フリーレン)</t>
         </is>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B10)</f>
         <v/>
       </c>
       <c r="E10" s="10">
+        <f>IF(D10&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F10" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B10,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F10" s="11">
+      <c r="G10" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B10,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G10" s="10">
+      <c r="H10" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B10,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H10" s="11">
+      <c r="I10" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B10,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I10" s="17">
+      <c r="J10" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B10)</f>
         <v/>
       </c>
-      <c r="J10" s="18">
+      <c r="K10" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B10)</f>
         <v/>
       </c>
@@ -8592,31 +9207,35 @@
           <t>葬送のフリーレンP　缶バッジ　(シュタルク)</t>
         </is>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B11)</f>
         <v/>
       </c>
       <c r="E11" s="10">
+        <f>IF(D11&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F11" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B11,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F11" s="11">
+      <c r="G11" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B11,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G11" s="10">
+      <c r="H11" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B11,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H11" s="11">
+      <c r="I11" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B11,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I11" s="17">
+      <c r="J11" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B11)</f>
         <v/>
       </c>
-      <c r="J11" s="18">
+      <c r="K11" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B11)</f>
         <v/>
       </c>
@@ -8637,31 +9256,35 @@
           <t>葬送のフリーレンP　缶バッジ　(フェルン)</t>
         </is>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B12)</f>
         <v/>
       </c>
       <c r="E12" s="10">
+        <f>IF(D12&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F12" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B12,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F12" s="11">
+      <c r="G12" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B12,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G12" s="10">
+      <c r="H12" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B12,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H12" s="11">
+      <c r="I12" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B12,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I12" s="17">
+      <c r="J12" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B12)</f>
         <v/>
       </c>
-      <c r="J12" s="18">
+      <c r="K12" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B12)</f>
         <v/>
       </c>
@@ -8682,31 +9305,35 @@
           <t>葬送のフリーレンP　フォトフレームキーホルダー　(フリーレン)</t>
         </is>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B13)</f>
         <v/>
       </c>
       <c r="E13" s="10">
+        <f>IF(D13&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F13" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B13,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F13" s="11">
+      <c r="G13" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B13,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G13" s="10">
+      <c r="H13" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B13,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H13" s="11">
+      <c r="I13" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B13,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I13" s="17">
+      <c r="J13" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B13)</f>
         <v/>
       </c>
-      <c r="J13" s="18">
+      <c r="K13" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B13)</f>
         <v/>
       </c>
@@ -8727,31 +9354,35 @@
           <t>葬送のフリーレンP　フォトフレームキーホルダー　(フェルン)</t>
         </is>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B14)</f>
         <v/>
       </c>
       <c r="E14" s="10">
+        <f>IF(D14&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F14" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B14,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F14" s="11">
+      <c r="G14" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B14,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G14" s="10">
+      <c r="H14" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B14,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H14" s="11">
+      <c r="I14" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B14,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I14" s="17">
+      <c r="J14" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B14)</f>
         <v/>
       </c>
-      <c r="J14" s="18">
+      <c r="K14" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B14)</f>
         <v/>
       </c>
@@ -8772,31 +9403,35 @@
           <t>葬送のフリーレンP　フォトフレームキーホルダー　(シュタルク)</t>
         </is>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B15)</f>
         <v/>
       </c>
       <c r="E15" s="10">
+        <f>IF(D15&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F15" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B15,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F15" s="11">
+      <c r="G15" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B15,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G15" s="10">
+      <c r="H15" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B15,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H15" s="11">
+      <c r="I15" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B15,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I15" s="17">
+      <c r="J15" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B15)</f>
         <v/>
       </c>
-      <c r="J15" s="18">
+      <c r="K15" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B15)</f>
         <v/>
       </c>
@@ -8817,31 +9452,35 @@
           <t>葬送のフリーレンP　ポストカードセット</t>
         </is>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B16)</f>
         <v/>
       </c>
       <c r="E16" s="10">
+        <f>IF(D16&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F16" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B16,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F16" s="11">
+      <c r="G16" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B16,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G16" s="10">
+      <c r="H16" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B16,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H16" s="11">
+      <c r="I16" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B16,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I16" s="17">
+      <c r="J16" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B16)</f>
         <v/>
       </c>
-      <c r="J16" s="18">
+      <c r="K16" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B16)</f>
         <v/>
       </c>
@@ -8862,31 +9501,35 @@
           <t>葬送のフリーレンP　ランダム魔導書風ノート　全6種</t>
         </is>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B17)</f>
         <v/>
       </c>
       <c r="E17" s="10">
+        <f>IF(D17&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F17" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B17,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F17" s="11">
+      <c r="G17" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B17,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G17" s="10">
+      <c r="H17" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B17,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H17" s="11">
+      <c r="I17" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B17,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I17" s="17">
+      <c r="J17" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B17)</f>
         <v/>
       </c>
-      <c r="J17" s="18">
+      <c r="K17" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B17)</f>
         <v/>
       </c>
@@ -8907,31 +9550,35 @@
           <t>葬送のフリーレンP　付箋</t>
         </is>
       </c>
-      <c r="D18" s="16">
+      <c r="D18" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B18)</f>
         <v/>
       </c>
       <c r="E18" s="10">
+        <f>IF(D18&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F18" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B18,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F18" s="11">
+      <c r="G18" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B18,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G18" s="10">
+      <c r="H18" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B18,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H18" s="11">
+      <c r="I18" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B18,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I18" s="17">
+      <c r="J18" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B18)</f>
         <v/>
       </c>
-      <c r="J18" s="18">
+      <c r="K18" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B18)</f>
         <v/>
       </c>
@@ -8952,31 +9599,35 @@
           <t>葬送のフリーレンP　ランダムパネルキーホルダー　全7種</t>
         </is>
       </c>
-      <c r="D19" s="16">
+      <c r="D19" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B19)</f>
         <v/>
       </c>
       <c r="E19" s="10">
+        <f>IF(D19&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F19" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B19,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F19" s="11">
+      <c r="G19" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B19,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G19" s="10">
+      <c r="H19" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B19,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H19" s="11">
+      <c r="I19" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B19,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I19" s="17">
+      <c r="J19" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B19)</f>
         <v/>
       </c>
-      <c r="J19" s="18">
+      <c r="K19" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B19)</f>
         <v/>
       </c>
@@ -8997,31 +9648,35 @@
           <t>ダンダダンPOPUP　クリアファイル　オカルン</t>
         </is>
       </c>
-      <c r="D20" s="16">
+      <c r="D20" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B20)</f>
         <v/>
       </c>
       <c r="E20" s="10">
+        <f>IF(D20&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F20" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B20,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F20" s="11">
+      <c r="G20" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B20,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G20" s="10">
+      <c r="H20" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B20,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H20" s="11">
+      <c r="I20" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B20,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I20" s="17">
+      <c r="J20" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B20)</f>
         <v/>
       </c>
-      <c r="J20" s="18">
+      <c r="K20" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B20)</f>
         <v/>
       </c>
@@ -9042,31 +9697,35 @@
           <t>ダンダダンPOPUP　クリアファイル　モモ</t>
         </is>
       </c>
-      <c r="D21" s="16">
+      <c r="D21" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B21)</f>
         <v/>
       </c>
       <c r="E21" s="10">
+        <f>IF(D21&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F21" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B21,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F21" s="11">
+      <c r="G21" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B21,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G21" s="10">
+      <c r="H21" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B21,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H21" s="11">
+      <c r="I21" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B21,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I21" s="17">
+      <c r="J21" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B21)</f>
         <v/>
       </c>
-      <c r="J21" s="18">
+      <c r="K21" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B21)</f>
         <v/>
       </c>
@@ -9087,31 +9746,35 @@
           <t>ダンダダンPOPUP　クリアファイル　星子</t>
         </is>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B22)</f>
         <v/>
       </c>
       <c r="E22" s="10">
+        <f>IF(D22&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F22" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B22,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F22" s="11">
+      <c r="G22" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B22,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G22" s="10">
+      <c r="H22" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B22,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H22" s="11">
+      <c r="I22" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B22,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I22" s="17">
+      <c r="J22" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B22)</f>
         <v/>
       </c>
-      <c r="J22" s="18">
+      <c r="K22" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B22)</f>
         <v/>
       </c>
@@ -9132,31 +9795,35 @@
           <t>ダンダダンPOPUP　クリアファイル　アイラ</t>
         </is>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B23)</f>
         <v/>
       </c>
       <c r="E23" s="10">
+        <f>IF(D23&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F23" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B23,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F23" s="11">
+      <c r="G23" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B23,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G23" s="10">
+      <c r="H23" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B23,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H23" s="11">
+      <c r="I23" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B23,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I23" s="17">
+      <c r="J23" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B23)</f>
         <v/>
       </c>
-      <c r="J23" s="18">
+      <c r="K23" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B23)</f>
         <v/>
       </c>
@@ -9177,31 +9844,35 @@
           <t>ダンダダンPOPUP　クリアファイル　ターボババア(招き猫)</t>
         </is>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B24)</f>
         <v/>
       </c>
       <c r="E24" s="10">
+        <f>IF(D24&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F24" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B24,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F24" s="11">
+      <c r="G24" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B24,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G24" s="10">
+      <c r="H24" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B24,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H24" s="11">
+      <c r="I24" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B24,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I24" s="17">
+      <c r="J24" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B24)</f>
         <v/>
       </c>
-      <c r="J24" s="18">
+      <c r="K24" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B24)</f>
         <v/>
       </c>
@@ -9222,31 +9893,35 @@
           <t>ダンダダンPOPUP　クリアファイル　オカルン(変身)</t>
         </is>
       </c>
-      <c r="D25" s="16">
+      <c r="D25" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B25)</f>
         <v/>
       </c>
       <c r="E25" s="10">
+        <f>IF(D25&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F25" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B25,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F25" s="11">
+      <c r="G25" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B25,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G25" s="10">
+      <c r="H25" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B25,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H25" s="11">
+      <c r="I25" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B25,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I25" s="17">
+      <c r="J25" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B25)</f>
         <v/>
       </c>
-      <c r="J25" s="18">
+      <c r="K25" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B25)</f>
         <v/>
       </c>
@@ -9267,31 +9942,35 @@
           <t>ダンダダンPOPUP　クリアファイル　アイラ(変身)</t>
         </is>
       </c>
-      <c r="D26" s="16">
+      <c r="D26" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B26)</f>
         <v/>
       </c>
       <c r="E26" s="10">
+        <f>IF(D26&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F26" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B26,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F26" s="11">
+      <c r="G26" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B26,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G26" s="10">
+      <c r="H26" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B26,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H26" s="11">
+      <c r="I26" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B26,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I26" s="17">
+      <c r="J26" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B26)</f>
         <v/>
       </c>
-      <c r="J26" s="18">
+      <c r="K26" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B26)</f>
         <v/>
       </c>
@@ -9312,31 +9991,35 @@
           <t>ダンダダンPOPUP　ランダム缶バッジ 全7種</t>
         </is>
       </c>
-      <c r="D27" s="16">
+      <c r="D27" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B27)</f>
         <v/>
       </c>
       <c r="E27" s="10">
+        <f>IF(D27&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F27" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B27,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F27" s="11">
+      <c r="G27" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B27,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G27" s="10">
+      <c r="H27" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B27,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H27" s="11">
+      <c r="I27" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B27,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I27" s="17">
+      <c r="J27" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B27)</f>
         <v/>
       </c>
-      <c r="J27" s="18">
+      <c r="K27" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B27)</f>
         <v/>
       </c>
@@ -9357,31 +10040,35 @@
           <t>ダンダダンPOPUP　アクリルスタンド　オカルン</t>
         </is>
       </c>
-      <c r="D28" s="16">
+      <c r="D28" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B28)</f>
         <v/>
       </c>
       <c r="E28" s="10">
+        <f>IF(D28&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F28" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B28,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F28" s="11">
+      <c r="G28" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B28,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G28" s="10">
+      <c r="H28" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B28,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H28" s="11">
+      <c r="I28" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B28,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I28" s="17">
+      <c r="J28" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B28)</f>
         <v/>
       </c>
-      <c r="J28" s="18">
+      <c r="K28" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B28)</f>
         <v/>
       </c>
@@ -9402,31 +10089,35 @@
           <t>ダンダダンPOPUP　アクリルスタンド　モモ</t>
         </is>
       </c>
-      <c r="D29" s="16">
+      <c r="D29" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B29)</f>
         <v/>
       </c>
       <c r="E29" s="10">
+        <f>IF(D29&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F29" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B29,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F29" s="11">
+      <c r="G29" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B29,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G29" s="10">
+      <c r="H29" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B29,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H29" s="11">
+      <c r="I29" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B29,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I29" s="17">
+      <c r="J29" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B29)</f>
         <v/>
       </c>
-      <c r="J29" s="18">
+      <c r="K29" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B29)</f>
         <v/>
       </c>
@@ -9447,31 +10138,35 @@
           <t>ダンダダンPOPUP　アクリルスタンド　星子</t>
         </is>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B30)</f>
         <v/>
       </c>
       <c r="E30" s="10">
+        <f>IF(D30&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F30" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B30,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F30" s="11">
+      <c r="G30" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B30,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G30" s="10">
+      <c r="H30" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B30,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H30" s="11">
+      <c r="I30" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B30,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I30" s="17">
+      <c r="J30" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B30)</f>
         <v/>
       </c>
-      <c r="J30" s="18">
+      <c r="K30" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B30)</f>
         <v/>
       </c>
@@ -9492,31 +10187,35 @@
           <t>ダンダダンPOPUP　アクリルスタンド　アイラ</t>
         </is>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B31)</f>
         <v/>
       </c>
       <c r="E31" s="10">
+        <f>IF(D31&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F31" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B31,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F31" s="11">
+      <c r="G31" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B31,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G31" s="10">
+      <c r="H31" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B31,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H31" s="11">
+      <c r="I31" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B31,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I31" s="17">
+      <c r="J31" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B31)</f>
         <v/>
       </c>
-      <c r="J31" s="18">
+      <c r="K31" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B31)</f>
         <v/>
       </c>
@@ -9537,31 +10236,35 @@
           <t>ダンダダンPOPUP　アクリルスタンド　ターボババア(招き猫)</t>
         </is>
       </c>
-      <c r="D32" s="16">
+      <c r="D32" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B32)</f>
         <v/>
       </c>
       <c r="E32" s="10">
+        <f>IF(D32&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F32" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B32,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F32" s="11">
+      <c r="G32" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B32,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G32" s="10">
+      <c r="H32" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B32,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H32" s="11">
+      <c r="I32" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B32,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I32" s="17">
+      <c r="J32" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B32)</f>
         <v/>
       </c>
-      <c r="J32" s="18">
+      <c r="K32" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B32)</f>
         <v/>
       </c>
@@ -9582,31 +10285,35 @@
           <t>ダンダダンPOPUP　アクリルスタンド　オカルン(変身)</t>
         </is>
       </c>
-      <c r="D33" s="16">
+      <c r="D33" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B33)</f>
         <v/>
       </c>
       <c r="E33" s="10">
+        <f>IF(D33&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F33" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B33,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F33" s="11">
+      <c r="G33" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B33,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G33" s="10">
+      <c r="H33" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B33,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H33" s="11">
+      <c r="I33" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B33,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I33" s="17">
+      <c r="J33" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B33)</f>
         <v/>
       </c>
-      <c r="J33" s="18">
+      <c r="K33" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B33)</f>
         <v/>
       </c>
@@ -9627,31 +10334,35 @@
           <t>ダンダダンPOPUP　アクリルスタンド　アイラ(変身)</t>
         </is>
       </c>
-      <c r="D34" s="16">
+      <c r="D34" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B34)</f>
         <v/>
       </c>
       <c r="E34" s="10">
+        <f>IF(D34&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F34" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B34,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F34" s="11">
+      <c r="G34" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B34,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G34" s="10">
+      <c r="H34" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B34,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H34" s="11">
+      <c r="I34" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B34,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I34" s="17">
+      <c r="J34" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B34)</f>
         <v/>
       </c>
-      <c r="J34" s="18">
+      <c r="K34" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B34)</f>
         <v/>
       </c>
@@ -9672,31 +10383,35 @@
           <t>ダンダダンPOPUP　ステッカー3枚セット　A</t>
         </is>
       </c>
-      <c r="D35" s="16">
+      <c r="D35" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B35)</f>
         <v/>
       </c>
       <c r="E35" s="10">
+        <f>IF(D35&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F35" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B35,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F35" s="11">
+      <c r="G35" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B35,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G35" s="10">
+      <c r="H35" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B35,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H35" s="11">
+      <c r="I35" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B35,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I35" s="17">
+      <c r="J35" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B35)</f>
         <v/>
       </c>
-      <c r="J35" s="18">
+      <c r="K35" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B35)</f>
         <v/>
       </c>
@@ -9717,31 +10432,35 @@
           <t>ダンダダンPOPUP　ステッカー3枚セット　B</t>
         </is>
       </c>
-      <c r="D36" s="16">
+      <c r="D36" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B36)</f>
         <v/>
       </c>
       <c r="E36" s="10">
+        <f>IF(D36&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F36" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B36,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F36" s="11">
+      <c r="G36" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B36,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G36" s="10">
+      <c r="H36" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B36,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H36" s="11">
+      <c r="I36" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B36,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I36" s="17">
+      <c r="J36" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B36)</f>
         <v/>
       </c>
-      <c r="J36" s="18">
+      <c r="K36" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B36)</f>
         <v/>
       </c>
@@ -9762,31 +10481,35 @@
           <t>ダンダダンPOPUP　ステッカー3枚セット　C</t>
         </is>
       </c>
-      <c r="D37" s="16">
+      <c r="D37" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B37)</f>
         <v/>
       </c>
       <c r="E37" s="10">
+        <f>IF(D37&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F37" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B37,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F37" s="11">
+      <c r="G37" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B37,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G37" s="10">
+      <c r="H37" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B37,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H37" s="11">
+      <c r="I37" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B37,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I37" s="17">
+      <c r="J37" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B37)</f>
         <v/>
       </c>
-      <c r="J37" s="18">
+      <c r="K37" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B37)</f>
         <v/>
       </c>
@@ -9807,31 +10530,35 @@
           <t>ダンダダンPOPUP　ランダム缶バッジ　オープニング　全6種</t>
         </is>
       </c>
-      <c r="D38" s="16">
+      <c r="D38" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B38)</f>
         <v/>
       </c>
       <c r="E38" s="10">
+        <f>IF(D38&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F38" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B38,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F38" s="11">
+      <c r="G38" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B38,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G38" s="10">
+      <c r="H38" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B38,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H38" s="11">
+      <c r="I38" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B38,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I38" s="17">
+      <c r="J38" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B38)</f>
         <v/>
       </c>
-      <c r="J38" s="18">
+      <c r="K38" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B38)</f>
         <v/>
       </c>
@@ -9852,31 +10579,35 @@
           <t>ダンダダンPOPUP　ランダム缶バッジ　エンディング　全6種</t>
         </is>
       </c>
-      <c r="D39" s="16">
+      <c r="D39" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B39)</f>
         <v/>
       </c>
       <c r="E39" s="10">
+        <f>IF(D39&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F39" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B39,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F39" s="11">
+      <c r="G39" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B39,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G39" s="10">
+      <c r="H39" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B39,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H39" s="11">
+      <c r="I39" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B39,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I39" s="17">
+      <c r="J39" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B39)</f>
         <v/>
       </c>
-      <c r="J39" s="18">
+      <c r="K39" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B39)</f>
         <v/>
       </c>
@@ -9897,31 +10628,35 @@
           <t>ダンダダンPOPUP　ランダムアクリルキーホルダー　全6種</t>
         </is>
       </c>
-      <c r="D40" s="16">
+      <c r="D40" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B40)</f>
         <v/>
       </c>
       <c r="E40" s="10">
+        <f>IF(D40&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F40" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B40,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F40" s="11">
+      <c r="G40" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B40,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G40" s="10">
+      <c r="H40" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B40,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H40" s="11">
+      <c r="I40" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B40,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I40" s="17">
+      <c r="J40" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B40)</f>
         <v/>
       </c>
-      <c r="J40" s="18">
+      <c r="K40" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B40)</f>
         <v/>
       </c>
@@ -9942,31 +10677,35 @@
           <t>ダンダダンPOPUP　トートバッグ</t>
         </is>
       </c>
-      <c r="D41" s="16">
+      <c r="D41" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B41)</f>
         <v/>
       </c>
       <c r="E41" s="10">
+        <f>IF(D41&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F41" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B41,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F41" s="11">
+      <c r="G41" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B41,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G41" s="10">
+      <c r="H41" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B41,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H41" s="11">
+      <c r="I41" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B41,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I41" s="17">
+      <c r="J41" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B41)</f>
         <v/>
       </c>
-      <c r="J41" s="18">
+      <c r="K41" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B41)</f>
         <v/>
       </c>
@@ -9987,31 +10726,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　オカルン(変身)</t>
         </is>
       </c>
-      <c r="D42" s="16">
+      <c r="D42" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B42)</f>
         <v/>
       </c>
       <c r="E42" s="10">
+        <f>IF(D42&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F42" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B42,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F42" s="11">
+      <c r="G42" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B42,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G42" s="10">
+      <c r="H42" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B42,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H42" s="11">
+      <c r="I42" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B42,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I42" s="17">
+      <c r="J42" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B42)</f>
         <v/>
       </c>
-      <c r="J42" s="18">
+      <c r="K42" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B42)</f>
         <v/>
       </c>
@@ -10032,31 +10775,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　モモ</t>
         </is>
       </c>
-      <c r="D43" s="16">
+      <c r="D43" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B43)</f>
         <v/>
       </c>
       <c r="E43" s="10">
+        <f>IF(D43&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F43" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B43,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F43" s="11">
+      <c r="G43" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B43,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G43" s="10">
+      <c r="H43" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B43,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H43" s="11">
+      <c r="I43" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B43,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I43" s="17">
+      <c r="J43" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B43)</f>
         <v/>
       </c>
-      <c r="J43" s="18">
+      <c r="K43" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B43)</f>
         <v/>
       </c>
@@ -10077,31 +10824,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　星子</t>
         </is>
       </c>
-      <c r="D44" s="16">
+      <c r="D44" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B44)</f>
         <v/>
       </c>
       <c r="E44" s="10">
+        <f>IF(D44&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F44" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B44,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F44" s="11">
+      <c r="G44" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B44,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G44" s="10">
+      <c r="H44" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B44,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H44" s="11">
+      <c r="I44" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B44,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I44" s="17">
+      <c r="J44" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B44)</f>
         <v/>
       </c>
-      <c r="J44" s="18">
+      <c r="K44" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B44)</f>
         <v/>
       </c>
@@ -10122,31 +10873,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　アイラ</t>
         </is>
       </c>
-      <c r="D45" s="16">
+      <c r="D45" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B45)</f>
         <v/>
       </c>
       <c r="E45" s="10">
+        <f>IF(D45&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F45" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B45,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F45" s="11">
+      <c r="G45" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B45,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G45" s="10">
+      <c r="H45" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B45,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H45" s="11">
+      <c r="I45" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B45,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I45" s="17">
+      <c r="J45" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B45)</f>
         <v/>
       </c>
-      <c r="J45" s="18">
+      <c r="K45" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B45)</f>
         <v/>
       </c>
@@ -10167,31 +10922,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　ジジ</t>
         </is>
       </c>
-      <c r="D46" s="16">
+      <c r="D46" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B46)</f>
         <v/>
       </c>
       <c r="E46" s="10">
+        <f>IF(D46&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F46" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B46,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F46" s="11">
+      <c r="G46" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B46,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G46" s="10">
+      <c r="H46" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B46,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H46" s="11">
+      <c r="I46" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B46,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I46" s="17">
+      <c r="J46" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B46)</f>
         <v/>
       </c>
-      <c r="J46" s="18">
+      <c r="K46" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B46)</f>
         <v/>
       </c>
@@ -10212,31 +10971,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　ターボババア(招き猫)</t>
         </is>
       </c>
-      <c r="D47" s="16">
+      <c r="D47" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B47)</f>
         <v/>
       </c>
       <c r="E47" s="10">
+        <f>IF(D47&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F47" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B47,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F47" s="11">
+      <c r="G47" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B47,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G47" s="10">
+      <c r="H47" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B47,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H47" s="11">
+      <c r="I47" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B47,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I47" s="17">
+      <c r="J47" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B47)</f>
         <v/>
       </c>
-      <c r="J47" s="18">
+      <c r="K47" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B47)</f>
         <v/>
       </c>
@@ -10257,31 +11020,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　セルポ星人</t>
         </is>
       </c>
-      <c r="D48" s="16">
+      <c r="D48" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B48)</f>
         <v/>
       </c>
       <c r="E48" s="10">
+        <f>IF(D48&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F48" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B48,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F48" s="11">
+      <c r="G48" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B48,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G48" s="10">
+      <c r="H48" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B48,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H48" s="11">
+      <c r="I48" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B48,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I48" s="17">
+      <c r="J48" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B48)</f>
         <v/>
       </c>
-      <c r="J48" s="18">
+      <c r="K48" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B48)</f>
         <v/>
       </c>
@@ -10302,31 +11069,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　アクロバティックさらさら</t>
         </is>
       </c>
-      <c r="D49" s="16">
+      <c r="D49" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B49)</f>
         <v/>
       </c>
       <c r="E49" s="10">
+        <f>IF(D49&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F49" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B49,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F49" s="11">
+      <c r="G49" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B49,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G49" s="10">
+      <c r="H49" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B49,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H49" s="11">
+      <c r="I49" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B49,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I49" s="17">
+      <c r="J49" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B49)</f>
         <v/>
       </c>
-      <c r="J49" s="18">
+      <c r="K49" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B49)</f>
         <v/>
       </c>
@@ -10347,31 +11118,35 @@
           <t>ダンダダンPOPUP　スライドアクリルキーホルダー　ドーバーデーモン</t>
         </is>
       </c>
-      <c r="D50" s="16">
+      <c r="D50" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B50)</f>
         <v/>
       </c>
       <c r="E50" s="10">
+        <f>IF(D50&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F50" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B50,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F50" s="11">
+      <c r="G50" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B50,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G50" s="10">
+      <c r="H50" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B50,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H50" s="11">
+      <c r="I50" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B50,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I50" s="17">
+      <c r="J50" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B50)</f>
         <v/>
       </c>
-      <c r="J50" s="18">
+      <c r="K50" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B50)</f>
         <v/>
       </c>
@@ -10392,31 +11167,35 @@
           <t>ダンダダンPOPUP　ランダムクリアカード＆ポストカードセット　全6種</t>
         </is>
       </c>
-      <c r="D51" s="16">
+      <c r="D51" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B51)</f>
         <v/>
       </c>
       <c r="E51" s="10">
+        <f>IF(D51&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F51" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B51,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F51" s="11">
+      <c r="G51" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B51,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G51" s="10">
+      <c r="H51" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B51,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H51" s="11">
+      <c r="I51" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B51,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I51" s="17">
+      <c r="J51" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B51)</f>
         <v/>
       </c>
-      <c r="J51" s="18">
+      <c r="K51" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B51)</f>
         <v/>
       </c>
@@ -10437,31 +11216,35 @@
           <t>ダンダダンPOPUP　ビジュアルポストカード　A</t>
         </is>
       </c>
-      <c r="D52" s="16">
+      <c r="D52" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B52)</f>
         <v/>
       </c>
       <c r="E52" s="10">
+        <f>IF(D52&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F52" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B52,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F52" s="11">
+      <c r="G52" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B52,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G52" s="10">
+      <c r="H52" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B52,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H52" s="11">
+      <c r="I52" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B52,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I52" s="17">
+      <c r="J52" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B52)</f>
         <v/>
       </c>
-      <c r="J52" s="18">
+      <c r="K52" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B52)</f>
         <v/>
       </c>
@@ -10482,78 +11265,202 @@
           <t>ダンダダンPOPUP　ビジュアルポストカード　B</t>
         </is>
       </c>
-      <c r="D53" s="16">
+      <c r="D53" s="10">
         <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B53)</f>
         <v/>
       </c>
       <c r="E53" s="10">
+        <f>IF(D53&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F53" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B53,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="F53" s="11">
+      <c r="G53" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B53,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
         <v/>
       </c>
-      <c r="G53" s="10">
+      <c r="H53" s="11">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B53,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="H53" s="11">
+      <c r="I53" s="12">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B53,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
         <v/>
       </c>
-      <c r="I53" s="17">
+      <c r="J53" s="25">
         <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B53)</f>
         <v/>
       </c>
-      <c r="J53" s="18">
+      <c r="K53" s="26">
         <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B53)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n"/>
-      <c r="B54" s="12" t="n"/>
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>QCX2412FRNPTFN-10</t>
+        </is>
+      </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
+          <t>葬送のフリーレンP 経費（課税10％）</t>
+        </is>
+      </c>
+      <c r="D54" s="14">
+        <f>COUNTIFS('XTab DS_1'!$B$2:$B$106,$B54)</f>
+        <v/>
+      </c>
+      <c r="E54" s="14">
+        <f>IF(D54&gt;=2,"重複","単独")</f>
+        <v/>
+      </c>
+      <c r="F54" s="15">
+        <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B54,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
+        <v/>
+      </c>
+      <c r="G54" s="16">
+        <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B54,'XTab DS_1'!$D$2:$D$106,"CX01")</f>
+        <v/>
+      </c>
+      <c r="H54" s="15">
+        <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B54,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
+        <v/>
+      </c>
+      <c r="I54" s="16">
+        <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B54,'XTab DS_1'!$D$2:$D$106,"DB00")</f>
+        <v/>
+      </c>
+      <c r="J54" s="27">
+        <f>SUMIFS('XTab DS_1'!$F$2:$F$106,'XTab DS_1'!$B$2:$B$106,$B54)</f>
+        <v/>
+      </c>
+      <c r="K54" s="28">
+        <f>SUMIFS('XTab DS_1'!$G$2:$G$106,'XTab DS_1'!$B$2:$B$106,$B54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="17" t="n"/>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D54" s="12" t="n"/>
-      <c r="E54" s="14">
-        <f>SUM(E2:E53)</f>
-        <v/>
-      </c>
-      <c r="F54" s="15">
-        <f>SUM(F2:F53)</f>
-        <v/>
-      </c>
-      <c r="G54" s="14">
-        <f>SUM(G2:G53)</f>
-        <v/>
-      </c>
-      <c r="H54" s="15">
-        <f>SUM(H2:H53)</f>
-        <v/>
-      </c>
-      <c r="I54" s="14">
-        <f>SUM(I2:I53)</f>
-        <v/>
-      </c>
-      <c r="J54" s="15">
-        <f>SUM(J2:J53)</f>
+      <c r="D55" s="17" t="n"/>
+      <c r="E55" s="17" t="n"/>
+      <c r="F55" s="19">
+        <f>SUM(F2:F54)</f>
+        <v/>
+      </c>
+      <c r="G55" s="20">
+        <f>SUM(G2:G54)</f>
+        <v/>
+      </c>
+      <c r="H55" s="19">
+        <f>SUM(H2:H54)</f>
+        <v/>
+      </c>
+      <c r="I55" s="20">
+        <f>SUM(I2:I54)</f>
+        <v/>
+      </c>
+      <c r="J55" s="19">
+        <f>SUM(J2:J54)</f>
+        <v/>
+      </c>
+      <c r="K55" s="20">
+        <f>SUM(K2:K54)</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="19" t="inlineStr">
-        <is>
-          <t>※元データ「XTab DS_1」から、2つ以上の倉庫(保管場所)に登録されている品目コードを抽出。数量・金額はSUMIFSで元データから集計（元データ変更で自動再計算）。</t>
+      <c r="A56" s="21" t="n"/>
+      <c r="B56" s="21" t="n"/>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>うち 重複</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="n"/>
+      <c r="E56" s="21" t="n"/>
+      <c r="F56" s="23">
+        <f>SUMIFS(F2:F54,E2:E54,"重複")</f>
+        <v/>
+      </c>
+      <c r="G56" s="24">
+        <f>SUMIFS(G2:G54,E2:E54,"重複")</f>
+        <v/>
+      </c>
+      <c r="H56" s="23">
+        <f>SUMIFS(H2:H54,E2:E54,"重複")</f>
+        <v/>
+      </c>
+      <c r="I56" s="24">
+        <f>SUMIFS(I2:I54,E2:E54,"重複")</f>
+        <v/>
+      </c>
+      <c r="J56" s="23">
+        <f>SUMIFS(J2:J54,E2:E54,"重複")</f>
+        <v/>
+      </c>
+      <c r="K56" s="24">
+        <f>SUMIFS(K2:K54,E2:E54,"重複")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="21" t="n"/>
+      <c r="B57" s="21" t="n"/>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>うち 単独</t>
+        </is>
+      </c>
+      <c r="D57" s="21" t="n"/>
+      <c r="E57" s="21" t="n"/>
+      <c r="F57" s="23">
+        <f>SUMIFS(F2:F54,E2:E54,"単独")</f>
+        <v/>
+      </c>
+      <c r="G57" s="24">
+        <f>SUMIFS(G2:G54,E2:E54,"単独")</f>
+        <v/>
+      </c>
+      <c r="H57" s="23">
+        <f>SUMIFS(H2:H54,E2:E54,"単独")</f>
+        <v/>
+      </c>
+      <c r="I57" s="24">
+        <f>SUMIFS(I2:I54,E2:E54,"単独")</f>
+        <v/>
+      </c>
+      <c r="J57" s="23">
+        <f>SUMIFS(J2:J54,E2:E54,"単独")</f>
+        <v/>
+      </c>
+      <c r="K57" s="24">
+        <f>SUMIFS(K2:K54,E2:E54,"単独")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="29" t="inlineStr">
+        <is>
+          <t>※元データ「XTab DS_1」の全品目を掲載。2つ以上の倉庫(保管場所)に登録されている品目を「重複」（黄色）、1倉庫のみを「単独」と表示。数量・金額はSUMIFSで元データから集計（元データ変更で自動再計算）。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:K54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>